<commit_message>
feat(4b_reclamos): seis reportes nuevos + insumos de la secretaria
reporte_deuda_ledger, reporte_seguimiento, reporte_convenio_multa (con su
auditor y el agregador de lotes), reporte_lote_saldo_negativo y
reporte_reimputacion_cascada: cada uno arma el PDF con el que se le explica
al vecino de donde sale su numero.

Suma inputs/, recursos/ y pendientes_secretaria/ (Grupo_1 y Grupo_2).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4b_reclamos/trazabilidad/trazabilidad_reclamos.xlsx
+++ b/4b_reclamos/trazabilidad/trazabilidad_reclamos.xlsx
@@ -605,7 +605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R36"/>
+  <dimension ref="A1:R87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3249,6 +3249,3396 @@
         <v>46190</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>mesa_1</t>
+        </is>
+      </c>
+      <c r="D37" s="10" t="inlineStr">
+        <is>
+          <t>Wilder</t>
+        </is>
+      </c>
+      <c r="E37" s="21" t="n">
+        <v>46176</v>
+      </c>
+      <c r="F37" s="22" t="n">
+        <v>38</v>
+      </c>
+      <c r="G37" s="13" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="H37" s="13" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="I37" s="14" t="inlineStr"/>
+      <c r="J37" s="15" t="inlineStr">
+        <is>
+          <t>reclamo A</t>
+        </is>
+      </c>
+      <c r="K37" s="15" t="inlineStr"/>
+      <c r="L37" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M37" s="17" t="inlineStr"/>
+      <c r="N37" s="18" t="n"/>
+      <c r="O37" s="18" t="n"/>
+      <c r="P37" s="23" t="n">
+        <v>46183</v>
+      </c>
+      <c r="Q37" s="20" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="R37" s="23" t="n">
+        <v>46223</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>mesa_2</t>
+        </is>
+      </c>
+      <c r="D38" s="10" t="inlineStr">
+        <is>
+          <t>Yerald</t>
+        </is>
+      </c>
+      <c r="E38" s="21" t="n">
+        <v>46177</v>
+      </c>
+      <c r="F38" s="22" t="n">
+        <v>44</v>
+      </c>
+      <c r="G38" s="13" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="H38" s="13" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="I38" s="14" t="inlineStr">
+        <is>
+          <t>convenio</t>
+        </is>
+      </c>
+      <c r="J38" s="15" t="inlineStr">
+        <is>
+          <t>reclamo B</t>
+        </is>
+      </c>
+      <c r="K38" s="15" t="inlineStr">
+        <is>
+          <t>deuda activa</t>
+        </is>
+      </c>
+      <c r="L38" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M38" s="17" t="inlineStr"/>
+      <c r="N38" s="18" t="n"/>
+      <c r="O38" s="18" t="n"/>
+      <c r="P38" s="23" t="n">
+        <v>46184</v>
+      </c>
+      <c r="Q38" s="20" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="R38" s="23" t="n">
+        <v>46223</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>mesa_1</t>
+        </is>
+      </c>
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>Wilder Trujillo Rosales</t>
+        </is>
+      </c>
+      <c r="E39" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F39" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="G39" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H39" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I39" s="14" t="inlineStr">
+        <is>
+          <t>convenio</t>
+        </is>
+      </c>
+      <c r="J39" s="15" t="inlineStr">
+        <is>
+          <t>Verificar convenio</t>
+        </is>
+      </c>
+      <c r="K39" s="15" t="inlineStr">
+        <is>
+          <t>Sin deuda convenio (SALDO ACTUAL=0) - error de boleta convenio ya corregido</t>
+        </is>
+      </c>
+      <c r="L39" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M39" s="17" t="inlineStr"/>
+      <c r="N39" s="18" t="n"/>
+      <c r="O39" s="18" t="n"/>
+      <c r="P39" s="23" t="n"/>
+      <c r="Q39" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R39" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>mesa_1</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="inlineStr">
+        <is>
+          <t>Wilder Trujillo Rosales</t>
+        </is>
+      </c>
+      <c r="E40" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F40" s="22" t="n">
+        <v>16</v>
+      </c>
+      <c r="G40" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H40" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I40" s="14" t="inlineStr"/>
+      <c r="J40" s="15" t="inlineStr">
+        <is>
+          <t>Ya pague multa 30</t>
+        </is>
+      </c>
+      <c r="K40" s="15" t="inlineStr">
+        <is>
+          <t>FUNDADO -- el pago (S/44 = 11 agua + 3 mant + 30 multa) quedo anotado por error en V-16 (mesa_5 junio f58, Maximo Encarnacion). Reasignado a V-6 via reidentificacion.xlsx, coincide exacto con el reclamo.</t>
+        </is>
+      </c>
+      <c r="L40" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M40" s="17" t="inlineStr"/>
+      <c r="N40" s="18" t="n"/>
+      <c r="O40" s="18" t="n"/>
+      <c r="P40" s="23" t="n">
+        <v>46224</v>
+      </c>
+      <c r="Q40" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R40" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>mesa_1</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>Wilder Trujillo Rosales</t>
+        </is>
+      </c>
+      <c r="E41" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F41" s="22" t="n">
+        <v>94</v>
+      </c>
+      <c r="G41" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H41" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I41" s="14" t="inlineStr">
+        <is>
+          <t>convenio</t>
+        </is>
+      </c>
+      <c r="J41" s="15" t="inlineStr">
+        <is>
+          <t>Revizar convenio</t>
+        </is>
+      </c>
+      <c r="K41" s="15" t="inlineStr">
+        <is>
+          <t>Sin deuda convenio (SALDO ACTUAL=0) - error de boleta convenio ya corregido</t>
+        </is>
+      </c>
+      <c r="L41" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M41" s="17" t="inlineStr"/>
+      <c r="N41" s="18" t="n"/>
+      <c r="O41" s="18" t="n"/>
+      <c r="P41" s="23" t="n"/>
+      <c r="Q41" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R41" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>mesa_1</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>Wilder Trujillo Rosales</t>
+        </is>
+      </c>
+      <c r="E42" s="21" t="n">
+        <v>46208</v>
+      </c>
+      <c r="F42" s="22" t="n">
+        <v>83</v>
+      </c>
+      <c r="G42" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H42" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I42" s="14" t="inlineStr"/>
+      <c r="J42" s="15" t="inlineStr">
+        <is>
+          <t>Reclamo. Consumo alto paga solo 8 no 38. Paga tambien techado campo 75.</t>
+        </is>
+      </c>
+      <c r="K42" s="15" t="inlineStr">
+        <is>
+          <t>Confirmado: techado/campo (75, nunca sembrado) + consumo corregido de 38 a 5 m3 (tarifa minima, orden directa de la secretaria, no disputa). Via genesis_tardia.xlsx + ajustes_cargo.xlsx. SALDO=0.</t>
+        </is>
+      </c>
+      <c r="L42" s="16" t="inlineStr">
+        <is>
+          <t>INFORMADO</t>
+        </is>
+      </c>
+      <c r="M42" s="17" t="inlineStr"/>
+      <c r="N42" s="18" t="n"/>
+      <c r="O42" s="18" t="n"/>
+      <c r="P42" s="23" t="n"/>
+      <c r="Q42" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R42" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>mesa_2</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>Yreald Romero</t>
+        </is>
+      </c>
+      <c r="E43" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F43" s="22" t="n">
+        <v>25</v>
+      </c>
+      <c r="G43" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H43" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I43" s="14" t="inlineStr"/>
+      <c r="J43" s="15" t="inlineStr">
+        <is>
+          <t>Modificar</t>
+        </is>
+      </c>
+      <c r="K43" s="15" t="inlineStr">
+        <is>
+          <t>reclamo sin detalle - sin deuda convenio - asumido error de boleta medidor</t>
+        </is>
+      </c>
+      <c r="L43" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M43" s="17" t="inlineStr"/>
+      <c r="N43" s="18" t="n"/>
+      <c r="O43" s="18" t="n"/>
+      <c r="P43" s="23" t="n"/>
+      <c r="Q43" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R43" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>mesa_2</t>
+        </is>
+      </c>
+      <c r="D44" s="10" t="inlineStr">
+        <is>
+          <t>Yreald Romero</t>
+        </is>
+      </c>
+      <c r="E44" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F44" s="22" t="n">
+        <v>16</v>
+      </c>
+      <c r="G44" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H44" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I44" s="14" t="inlineStr"/>
+      <c r="J44" s="15" t="inlineStr">
+        <is>
+          <t>Modificar</t>
+        </is>
+      </c>
+      <c r="K44" s="15" t="inlineStr">
+        <is>
+          <t>reclamo sin detalle - sin deuda convenio - asumido error de boleta medidor</t>
+        </is>
+      </c>
+      <c r="L44" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M44" s="17" t="inlineStr"/>
+      <c r="N44" s="18" t="n"/>
+      <c r="O44" s="18" t="n"/>
+      <c r="P44" s="23" t="n"/>
+      <c r="Q44" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R44" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>mesa_2</t>
+        </is>
+      </c>
+      <c r="D45" s="10" t="inlineStr">
+        <is>
+          <t>Yreald Romero</t>
+        </is>
+      </c>
+      <c r="E45" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F45" s="22" t="n">
+        <v>22</v>
+      </c>
+      <c r="G45" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H45" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I45" s="14" t="inlineStr"/>
+      <c r="J45" s="15" t="inlineStr">
+        <is>
+          <t>Modificar</t>
+        </is>
+      </c>
+      <c r="K45" s="15" t="inlineStr">
+        <is>
+          <t>reclamo sin detalle - sin deuda convenio - asumido error de boleta medidor</t>
+        </is>
+      </c>
+      <c r="L45" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M45" s="17" t="inlineStr"/>
+      <c r="N45" s="18" t="n"/>
+      <c r="O45" s="18" t="n"/>
+      <c r="P45" s="23" t="n"/>
+      <c r="Q45" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R45" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>mesa_2</t>
+        </is>
+      </c>
+      <c r="D46" s="10" t="inlineStr">
+        <is>
+          <t>Yreald Romero</t>
+        </is>
+      </c>
+      <c r="E46" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F46" s="22" t="n">
+        <v>27</v>
+      </c>
+      <c r="G46" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H46" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I46" s="14" t="inlineStr"/>
+      <c r="J46" s="15" t="inlineStr">
+        <is>
+          <t>Modificar</t>
+        </is>
+      </c>
+      <c r="K46" s="15" t="inlineStr">
+        <is>
+          <t>reclamo sin detalle - sin deuda convenio - asumido error de boleta medidor</t>
+        </is>
+      </c>
+      <c r="L46" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M46" s="17" t="inlineStr"/>
+      <c r="N46" s="18" t="n"/>
+      <c r="O46" s="18" t="n"/>
+      <c r="P46" s="23" t="n"/>
+      <c r="Q46" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R46" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>mesa_2</t>
+        </is>
+      </c>
+      <c r="D47" s="10" t="inlineStr">
+        <is>
+          <t>Yreald Romero</t>
+        </is>
+      </c>
+      <c r="E47" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F47" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G47" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H47" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I47" s="14" t="inlineStr"/>
+      <c r="J47" s="15" t="inlineStr">
+        <is>
+          <t>Modificar</t>
+        </is>
+      </c>
+      <c r="K47" s="15" t="inlineStr">
+        <is>
+          <t>reclamo sin detalle - sin deuda convenio - asumido error de boleta medidor</t>
+        </is>
+      </c>
+      <c r="L47" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M47" s="17" t="inlineStr"/>
+      <c r="N47" s="18" t="n"/>
+      <c r="O47" s="18" t="n"/>
+      <c r="P47" s="23" t="n"/>
+      <c r="Q47" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R47" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>mesa_2</t>
+        </is>
+      </c>
+      <c r="D48" s="10" t="inlineStr">
+        <is>
+          <t>Yreald Romero</t>
+        </is>
+      </c>
+      <c r="E48" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F48" s="22" t="n">
+        <v>16</v>
+      </c>
+      <c r="G48" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H48" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I48" s="14" t="inlineStr"/>
+      <c r="J48" s="15" t="inlineStr">
+        <is>
+          <t>Modificar</t>
+        </is>
+      </c>
+      <c r="K48" s="15" t="inlineStr">
+        <is>
+          <t>reclamo sin detalle - sin deuda convenio - asumido error de boleta medidor</t>
+        </is>
+      </c>
+      <c r="L48" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M48" s="17" t="inlineStr"/>
+      <c r="N48" s="18" t="n"/>
+      <c r="O48" s="18" t="n"/>
+      <c r="P48" s="23" t="n"/>
+      <c r="Q48" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R48" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="inlineStr">
+        <is>
+          <t>mesa_2</t>
+        </is>
+      </c>
+      <c r="D49" s="10" t="inlineStr">
+        <is>
+          <t>Yreald Romero</t>
+        </is>
+      </c>
+      <c r="E49" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F49" s="22" t="n">
+        <v>45</v>
+      </c>
+      <c r="G49" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H49" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I49" s="14" t="inlineStr"/>
+      <c r="J49" s="15" t="inlineStr">
+        <is>
+          <t>Modificar</t>
+        </is>
+      </c>
+      <c r="K49" s="15" t="inlineStr">
+        <is>
+          <t>reclamo sin detalle - sin deuda convenio - asumido error de boleta medidor</t>
+        </is>
+      </c>
+      <c r="L49" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M49" s="17" t="inlineStr"/>
+      <c r="N49" s="18" t="n"/>
+      <c r="O49" s="18" t="n"/>
+      <c r="P49" s="23" t="n"/>
+      <c r="Q49" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R49" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>mesa_2</t>
+        </is>
+      </c>
+      <c r="D50" s="10" t="inlineStr">
+        <is>
+          <t>Yreald Romero</t>
+        </is>
+      </c>
+      <c r="E50" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F50" s="22" t="n">
+        <v>29</v>
+      </c>
+      <c r="G50" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H50" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I50" s="14" t="inlineStr"/>
+      <c r="J50" s="15" t="inlineStr">
+        <is>
+          <t>Modificar</t>
+        </is>
+      </c>
+      <c r="K50" s="15" t="inlineStr">
+        <is>
+          <t>reclamo sin detalle - sin deuda convenio - asumido error de boleta medidor</t>
+        </is>
+      </c>
+      <c r="L50" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M50" s="17" t="inlineStr"/>
+      <c r="N50" s="18" t="n"/>
+      <c r="O50" s="18" t="n"/>
+      <c r="P50" s="23" t="n"/>
+      <c r="Q50" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R50" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr">
+        <is>
+          <t>mesa_2</t>
+        </is>
+      </c>
+      <c r="D51" s="10" t="inlineStr">
+        <is>
+          <t>Yreald Romero</t>
+        </is>
+      </c>
+      <c r="E51" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F51" s="22" t="n">
+        <v>13</v>
+      </c>
+      <c r="G51" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H51" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I51" s="14" t="inlineStr"/>
+      <c r="J51" s="15" t="inlineStr">
+        <is>
+          <t>Modificar</t>
+        </is>
+      </c>
+      <c r="K51" s="15" t="inlineStr">
+        <is>
+          <t>reclamo sin detalle - sin deuda convenio - asumido error de boleta medidor</t>
+        </is>
+      </c>
+      <c r="L51" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M51" s="17" t="inlineStr"/>
+      <c r="N51" s="18" t="n"/>
+      <c r="O51" s="18" t="n"/>
+      <c r="P51" s="23" t="n"/>
+      <c r="Q51" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R51" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B52" s="8" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>mesa_4</t>
+        </is>
+      </c>
+      <c r="D52" s="10" t="inlineStr">
+        <is>
+          <t>Wagner Trujillo</t>
+        </is>
+      </c>
+      <c r="E52" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F52" s="22" t="n">
+        <v>9</v>
+      </c>
+      <c r="G52" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H52" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I52" s="14" t="inlineStr">
+        <is>
+          <t>convenio</t>
+        </is>
+      </c>
+      <c r="J52" s="15" t="inlineStr">
+        <is>
+          <t>Corregir convenio medidor</t>
+        </is>
+      </c>
+      <c r="K52" s="15" t="inlineStr">
+        <is>
+          <t>Sin deuda convenio (SALDO ACTUAL=0) - error de boleta convenio ya corregido</t>
+        </is>
+      </c>
+      <c r="L52" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M52" s="17" t="inlineStr"/>
+      <c r="N52" s="18" t="n"/>
+      <c r="O52" s="18" t="n"/>
+      <c r="P52" s="23" t="n"/>
+      <c r="Q52" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R52" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr">
+        <is>
+          <t>mesa_4</t>
+        </is>
+      </c>
+      <c r="D53" s="10" t="inlineStr">
+        <is>
+          <t>Wagner Trujillo</t>
+        </is>
+      </c>
+      <c r="E53" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F53" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G53" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H53" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I53" s="14" t="inlineStr">
+        <is>
+          <t>convenio</t>
+        </is>
+      </c>
+      <c r="J53" s="15" t="inlineStr">
+        <is>
+          <t>Corregir convenio medidor</t>
+        </is>
+      </c>
+      <c r="K53" s="15" t="inlineStr">
+        <is>
+          <t>Sin deuda convenio (SALDO ACTUAL=0) - error de boleta convenio ya corregido</t>
+        </is>
+      </c>
+      <c r="L53" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M53" s="17" t="inlineStr"/>
+      <c r="N53" s="18" t="n"/>
+      <c r="O53" s="18" t="n"/>
+      <c r="P53" s="23" t="n"/>
+      <c r="Q53" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R53" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>mesa_4</t>
+        </is>
+      </c>
+      <c r="D54" s="10" t="inlineStr">
+        <is>
+          <t>Wagner Trujillo</t>
+        </is>
+      </c>
+      <c r="E54" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F54" s="22" t="n">
+        <v>25</v>
+      </c>
+      <c r="G54" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H54" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I54" s="14" t="inlineStr"/>
+      <c r="J54" s="15" t="inlineStr">
+        <is>
+          <t>Coreccion</t>
+        </is>
+      </c>
+      <c r="K54" s="15" t="inlineStr">
+        <is>
+          <t>reclamo sin detalle - sin deuda convenio - asumido error de boleta medidor</t>
+        </is>
+      </c>
+      <c r="L54" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M54" s="17" t="inlineStr"/>
+      <c r="N54" s="18" t="n"/>
+      <c r="O54" s="18" t="n"/>
+      <c r="P54" s="23" t="n"/>
+      <c r="Q54" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R54" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="B55" s="8" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C55" s="9" t="inlineStr">
+        <is>
+          <t>mesa_4</t>
+        </is>
+      </c>
+      <c r="D55" s="10" t="inlineStr">
+        <is>
+          <t>Wagner Trujillo</t>
+        </is>
+      </c>
+      <c r="E55" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F55" s="22" t="n">
+        <v>44</v>
+      </c>
+      <c r="G55" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H55" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I55" s="14" t="inlineStr"/>
+      <c r="J55" s="15" t="inlineStr">
+        <is>
+          <t>Coreccion</t>
+        </is>
+      </c>
+      <c r="K55" s="15" t="inlineStr">
+        <is>
+          <t>reclamo sin detalle - sin deuda convenio - asumido error de boleta medidor</t>
+        </is>
+      </c>
+      <c r="L55" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M55" s="17" t="inlineStr"/>
+      <c r="N55" s="18" t="n"/>
+      <c r="O55" s="18" t="n"/>
+      <c r="P55" s="23" t="n"/>
+      <c r="Q55" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R55" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr">
+        <is>
+          <t>mesa_4</t>
+        </is>
+      </c>
+      <c r="D56" s="10" t="inlineStr">
+        <is>
+          <t>Wagner Trujillo</t>
+        </is>
+      </c>
+      <c r="E56" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F56" s="22" t="n">
+        <v>39</v>
+      </c>
+      <c r="G56" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H56" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I56" s="14" t="inlineStr">
+        <is>
+          <t>convenio</t>
+        </is>
+      </c>
+      <c r="J56" s="15" t="inlineStr">
+        <is>
+          <t>Correccion medidor</t>
+        </is>
+      </c>
+      <c r="K56" s="15" t="inlineStr">
+        <is>
+          <t>Sin deuda convenio (SALDO ACTUAL=0) - error de boleta convenio ya corregido</t>
+        </is>
+      </c>
+      <c r="L56" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M56" s="17" t="inlineStr"/>
+      <c r="N56" s="18" t="n"/>
+      <c r="O56" s="18" t="n"/>
+      <c r="P56" s="23" t="n"/>
+      <c r="Q56" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R56" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="C57" s="9" t="inlineStr">
+        <is>
+          <t>mesa_4</t>
+        </is>
+      </c>
+      <c r="D57" s="10" t="inlineStr">
+        <is>
+          <t>Wagner Trujillo</t>
+        </is>
+      </c>
+      <c r="E57" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F57" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G57" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H57" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I57" s="14" t="inlineStr">
+        <is>
+          <t>convenio</t>
+        </is>
+      </c>
+      <c r="J57" s="15" t="inlineStr">
+        <is>
+          <t>Correccion medidor</t>
+        </is>
+      </c>
+      <c r="K57" s="15" t="inlineStr">
+        <is>
+          <t>Sin deuda convenio (SALDO ACTUAL=0) - error de boleta convenio ya corregido</t>
+        </is>
+      </c>
+      <c r="L57" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M57" s="17" t="inlineStr"/>
+      <c r="N57" s="18" t="n"/>
+      <c r="O57" s="18" t="n"/>
+      <c r="P57" s="23" t="n"/>
+      <c r="Q57" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R57" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B58" s="8" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C58" s="9" t="inlineStr">
+        <is>
+          <t>mesa_4</t>
+        </is>
+      </c>
+      <c r="D58" s="10" t="inlineStr">
+        <is>
+          <t>Wagner Trujillo</t>
+        </is>
+      </c>
+      <c r="E58" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F58" s="22" t="n">
+        <v>83</v>
+      </c>
+      <c r="G58" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H58" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I58" s="14" t="inlineStr">
+        <is>
+          <t>convenio</t>
+        </is>
+      </c>
+      <c r="J58" s="15" t="inlineStr">
+        <is>
+          <t>Pago ultimo mes medidor</t>
+        </is>
+      </c>
+      <c r="K58" s="15" t="inlineStr">
+        <is>
+          <t>Sin deuda convenio (SALDO ACTUAL=0) - error de boleta convenio ya corregido</t>
+        </is>
+      </c>
+      <c r="L58" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M58" s="17" t="inlineStr"/>
+      <c r="N58" s="18" t="n"/>
+      <c r="O58" s="18" t="n"/>
+      <c r="P58" s="23" t="n"/>
+      <c r="Q58" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R58" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B59" s="8" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr">
+        <is>
+          <t>mesa_4</t>
+        </is>
+      </c>
+      <c r="D59" s="10" t="inlineStr">
+        <is>
+          <t>Wagner Trujillo</t>
+        </is>
+      </c>
+      <c r="E59" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F59" s="22" t="n">
+        <v>63</v>
+      </c>
+      <c r="G59" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H59" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I59" s="14" t="inlineStr">
+        <is>
+          <t>convenio</t>
+        </is>
+      </c>
+      <c r="J59" s="15" t="inlineStr">
+        <is>
+          <t>Revizar lectura de medidor</t>
+        </is>
+      </c>
+      <c r="K59" s="15" t="inlineStr">
+        <is>
+          <t>Sin deuda convenio (SALDO ACTUAL=0) - error de boleta convenio ya corregido</t>
+        </is>
+      </c>
+      <c r="L59" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M59" s="17" t="inlineStr"/>
+      <c r="N59" s="18" t="n"/>
+      <c r="O59" s="18" t="n"/>
+      <c r="P59" s="23" t="n"/>
+      <c r="Q59" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R59" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C60" s="9" t="inlineStr">
+        <is>
+          <t>mesa_4</t>
+        </is>
+      </c>
+      <c r="D60" s="10" t="inlineStr">
+        <is>
+          <t>Wagner Trujillo</t>
+        </is>
+      </c>
+      <c r="E60" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F60" s="22" t="n">
+        <v>20</v>
+      </c>
+      <c r="G60" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H60" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I60" s="14" t="inlineStr">
+        <is>
+          <t>convenio</t>
+        </is>
+      </c>
+      <c r="J60" s="15" t="inlineStr">
+        <is>
+          <t>Cambio de medidor observar</t>
+        </is>
+      </c>
+      <c r="K60" s="15" t="inlineStr">
+        <is>
+          <t>No tiene convenio en ledger - error de boleta convenio ya corregido</t>
+        </is>
+      </c>
+      <c r="L60" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M60" s="17" t="inlineStr"/>
+      <c r="N60" s="18" t="n"/>
+      <c r="O60" s="18" t="n"/>
+      <c r="P60" s="23" t="n"/>
+      <c r="Q60" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R60" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B61" s="8" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C61" s="9" t="inlineStr">
+        <is>
+          <t>mesa_4</t>
+        </is>
+      </c>
+      <c r="D61" s="10" t="inlineStr">
+        <is>
+          <t>Wagner Trujillo</t>
+        </is>
+      </c>
+      <c r="E61" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F61" s="22" t="n">
+        <v>20</v>
+      </c>
+      <c r="G61" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H61" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I61" s="14" t="inlineStr">
+        <is>
+          <t>convenio</t>
+        </is>
+      </c>
+      <c r="J61" s="15" t="inlineStr">
+        <is>
+          <t>Observar rectifica medidor</t>
+        </is>
+      </c>
+      <c r="K61" s="15" t="inlineStr">
+        <is>
+          <t>Sin deuda convenio (SALDO ACTUAL=0) - error de boleta convenio ya corregido</t>
+        </is>
+      </c>
+      <c r="L61" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M61" s="17" t="inlineStr"/>
+      <c r="N61" s="18" t="n"/>
+      <c r="O61" s="18" t="n"/>
+      <c r="P61" s="23" t="n"/>
+      <c r="Q61" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R61" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="B62" s="8" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C62" s="9" t="inlineStr">
+        <is>
+          <t>mesa_4</t>
+        </is>
+      </c>
+      <c r="D62" s="10" t="inlineStr">
+        <is>
+          <t>Wagner Trujillo</t>
+        </is>
+      </c>
+      <c r="E62" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F62" s="22" t="n">
+        <v>38</v>
+      </c>
+      <c r="G62" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H62" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I62" s="14" t="inlineStr">
+        <is>
+          <t>convenio</t>
+        </is>
+      </c>
+      <c r="J62" s="15" t="inlineStr">
+        <is>
+          <t>Cancelo convenio</t>
+        </is>
+      </c>
+      <c r="K62" s="15" t="inlineStr">
+        <is>
+          <t>No tiene convenio en ledger - error de boleta convenio ya corregido</t>
+        </is>
+      </c>
+      <c r="L62" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M62" s="17" t="inlineStr"/>
+      <c r="N62" s="18" t="n"/>
+      <c r="O62" s="18" t="n"/>
+      <c r="P62" s="23" t="n"/>
+      <c r="Q62" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R62" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="B63" s="8" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C63" s="9" t="inlineStr">
+        <is>
+          <t>mesa_4</t>
+        </is>
+      </c>
+      <c r="D63" s="10" t="inlineStr">
+        <is>
+          <t>Wagner Trujillo</t>
+        </is>
+      </c>
+      <c r="E63" s="21" t="n">
+        <v>46208</v>
+      </c>
+      <c r="F63" s="22" t="n">
+        <v>36</v>
+      </c>
+      <c r="G63" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H63" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I63" s="14" t="inlineStr">
+        <is>
+          <t>convenio</t>
+        </is>
+      </c>
+      <c r="J63" s="15" t="inlineStr">
+        <is>
+          <t>Reclamo. Correccion medidor</t>
+        </is>
+      </c>
+      <c r="K63" s="15" t="inlineStr">
+        <is>
+          <t>Sin deuda convenio (SALDO ACTUAL=0) - error de boleta convenio ya corregido</t>
+        </is>
+      </c>
+      <c r="L63" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M63" s="17" t="inlineStr"/>
+      <c r="N63" s="18" t="n"/>
+      <c r="O63" s="18" t="n"/>
+      <c r="P63" s="23" t="n"/>
+      <c r="Q63" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R63" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="B64" s="8" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C64" s="9" t="inlineStr">
+        <is>
+          <t>mesa_4</t>
+        </is>
+      </c>
+      <c r="D64" s="10" t="inlineStr">
+        <is>
+          <t>Wagner Trujillo</t>
+        </is>
+      </c>
+      <c r="E64" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F64" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H64" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I64" s="14" t="inlineStr">
+        <is>
+          <t>convenio</t>
+        </is>
+      </c>
+      <c r="J64" s="15" t="inlineStr">
+        <is>
+          <t>Cancelo medidor</t>
+        </is>
+      </c>
+      <c r="K64" s="15" t="inlineStr">
+        <is>
+          <t>Sin deuda convenio (SALDO ACTUAL=0) - error de boleta convenio ya corregido</t>
+        </is>
+      </c>
+      <c r="L64" s="16" t="inlineStr">
+        <is>
+          <t>RECHAZADO</t>
+        </is>
+      </c>
+      <c r="M64" s="17" t="inlineStr"/>
+      <c r="N64" s="18" t="n"/>
+      <c r="O64" s="18" t="n"/>
+      <c r="P64" s="23" t="n"/>
+      <c r="Q64" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R64" s="23" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B65" s="8" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C65" s="9" t="inlineStr">
+        <is>
+          <t>mesa_1</t>
+        </is>
+      </c>
+      <c r="D65" s="10" t="inlineStr">
+        <is>
+          <t>Wilder Trujillo Rosales</t>
+        </is>
+      </c>
+      <c r="E65" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F65" s="22" t="n">
+        <v>28</v>
+      </c>
+      <c r="G65" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H65" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I65" s="14" t="inlineStr"/>
+      <c r="J65" s="15" t="inlineStr">
+        <is>
+          <t>Cambiar la multa de G1-M15</t>
+        </is>
+      </c>
+      <c r="K65" s="15" t="inlineStr">
+        <is>
+          <t>Confirmado: M-15 pago de mas cubria la multa de G-1 por error del cobrador (misma fecha/cobrador). Reasignado via shared/reidentificacion.xlsx. G-1 SALDO=0 CANCELADO; M-15 queda con exceso de 20 a su favor (SALDO=-20).</t>
+        </is>
+      </c>
+      <c r="L65" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M65" s="17" t="inlineStr"/>
+      <c r="N65" s="18" t="n"/>
+      <c r="O65" s="18" t="n"/>
+      <c r="P65" s="23" t="n">
+        <v>46227.61004721065</v>
+      </c>
+      <c r="Q65" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R65" s="23" t="n">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B66" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C66" s="9" t="inlineStr">
+        <is>
+          <t>mesa_1</t>
+        </is>
+      </c>
+      <c r="D66" s="10" t="inlineStr">
+        <is>
+          <t>Wilder Trujillo Rosales</t>
+        </is>
+      </c>
+      <c r="E66" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F66" s="22" t="n">
+        <v>25</v>
+      </c>
+      <c r="G66" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H66" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I66" s="14" t="inlineStr"/>
+      <c r="J66" s="15" t="inlineStr">
+        <is>
+          <t>Cambiar la multa de G1-M15</t>
+        </is>
+      </c>
+      <c r="K66" s="15" t="inlineStr">
+        <is>
+          <t>Confirmado: le faltaban exactos 20 de multa que M-15 habia pagado de mas por error del cobrador. Reasignado via shared/reidentificacion.xlsx. SALDO=0 CANCELADO.</t>
+        </is>
+      </c>
+      <c r="L66" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M66" s="17" t="inlineStr"/>
+      <c r="N66" s="18" t="n"/>
+      <c r="O66" s="18" t="n"/>
+      <c r="P66" s="23" t="n">
+        <v>46227.61004721065</v>
+      </c>
+      <c r="Q66" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R66" s="23" t="n">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B67" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C67" s="9" t="inlineStr">
+        <is>
+          <t>mesa_1</t>
+        </is>
+      </c>
+      <c r="D67" s="10" t="inlineStr">
+        <is>
+          <t>Wilder Trujillo Rosales</t>
+        </is>
+      </c>
+      <c r="E67" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F67" s="22" t="n">
+        <v>22</v>
+      </c>
+      <c r="G67" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H67" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I67" s="14" t="inlineStr"/>
+      <c r="J67" s="15" t="inlineStr">
+        <is>
+          <t>937 518 732</t>
+        </is>
+      </c>
+      <c r="K67" s="15" t="inlineStr"/>
+      <c r="L67" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M67" s="17" t="inlineStr"/>
+      <c r="N67" s="18" t="n"/>
+      <c r="O67" s="18" t="n"/>
+      <c r="P67" s="23" t="n"/>
+      <c r="Q67" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R67" s="23" t="n">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B68" s="8" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C68" s="9" t="inlineStr">
+        <is>
+          <t>mesa_1</t>
+        </is>
+      </c>
+      <c r="D68" s="10" t="inlineStr">
+        <is>
+          <t>Wilder Trujillo Rosales</t>
+        </is>
+      </c>
+      <c r="E68" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F68" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G68" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H68" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I68" s="14" t="inlineStr">
+        <is>
+          <t>mes_anterior</t>
+        </is>
+      </c>
+      <c r="J68" s="15" t="inlineStr">
+        <is>
+          <t>Tiene exesa cancelo 58 mes pasado esta al dia.</t>
+        </is>
+      </c>
+      <c r="K68" s="15" t="inlineStr">
+        <is>
+          <t>Confirmado: exceso de junio (pago 58, debia 33) se aplico a su convenio/medidor via shared/devoluciones_aplicadas.xlsx. SALDO=0 CANCELADO, esta al dia como decia.</t>
+        </is>
+      </c>
+      <c r="L68" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M68" s="17" t="inlineStr"/>
+      <c r="N68" s="18" t="n"/>
+      <c r="O68" s="18" t="n"/>
+      <c r="P68" s="23" t="n">
+        <v>46227.61004721065</v>
+      </c>
+      <c r="Q68" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R68" s="23" t="n">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B69" s="8" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C69" s="9" t="inlineStr">
+        <is>
+          <t>mesa_1</t>
+        </is>
+      </c>
+      <c r="D69" s="10" t="inlineStr">
+        <is>
+          <t>Wilder Trujillo Rosales</t>
+        </is>
+      </c>
+      <c r="E69" s="21" t="n">
+        <v>46208</v>
+      </c>
+      <c r="F69" s="22" t="n">
+        <v>21</v>
+      </c>
+      <c r="G69" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H69" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I69" s="14" t="inlineStr"/>
+      <c r="J69" s="15" t="inlineStr">
+        <is>
+          <t>Reclamo. Cambiar mi apellido esta al revez.</t>
+        </is>
+      </c>
+      <c r="K69" s="15" t="inlineStr"/>
+      <c r="L69" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M69" s="17" t="inlineStr"/>
+      <c r="N69" s="18" t="n"/>
+      <c r="O69" s="18" t="n"/>
+      <c r="P69" s="23" t="n"/>
+      <c r="Q69" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R69" s="23" t="n">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="B70" s="8" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C70" s="9" t="inlineStr">
+        <is>
+          <t>mesa_1</t>
+        </is>
+      </c>
+      <c r="D70" s="10" t="inlineStr">
+        <is>
+          <t>Wilder Trujillo Rosales</t>
+        </is>
+      </c>
+      <c r="E70" s="21" t="n">
+        <v>46208</v>
+      </c>
+      <c r="F70" s="22" t="n">
+        <v>9</v>
+      </c>
+      <c r="G70" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H70" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I70" s="14" t="inlineStr">
+        <is>
+          <t>mes_anterior</t>
+        </is>
+      </c>
+      <c r="J70" s="15" t="inlineStr">
+        <is>
+          <t>Reclamo. Ya pague mes anterior 18.5. Pague faena. Cambiar mz: C1-17 a C1-9</t>
+        </is>
+      </c>
+      <c r="K70" s="15" t="inlineStr"/>
+      <c r="L70" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M70" s="17" t="inlineStr"/>
+      <c r="N70" s="18" t="n"/>
+      <c r="O70" s="18" t="n"/>
+      <c r="P70" s="23" t="n"/>
+      <c r="Q70" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R70" s="23" t="n">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B71" s="8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C71" s="9" t="inlineStr">
+        <is>
+          <t>mesa_2</t>
+        </is>
+      </c>
+      <c r="D71" s="10" t="inlineStr">
+        <is>
+          <t>Yreald Romero</t>
+        </is>
+      </c>
+      <c r="E71" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F71" s="22" t="n">
+        <v>18</v>
+      </c>
+      <c r="G71" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H71" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I71" s="14" t="inlineStr">
+        <is>
+          <t>mes_anterior</t>
+        </is>
+      </c>
+      <c r="J71" s="15" t="inlineStr">
+        <is>
+          <t>Modificar 24/06/2026</t>
+        </is>
+      </c>
+      <c r="K71" s="15" t="inlineStr">
+        <is>
+          <t>Su pago estaba como blanco en Junio</t>
+        </is>
+      </c>
+      <c r="L71" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M71" s="17" t="inlineStr"/>
+      <c r="N71" s="18" t="n"/>
+      <c r="O71" s="18" t="n"/>
+      <c r="P71" s="23" t="n"/>
+      <c r="Q71" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R71" s="23" t="n">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="8" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="B72" s="8" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C72" s="9" t="inlineStr">
+        <is>
+          <t>mesa_3</t>
+        </is>
+      </c>
+      <c r="D72" s="10" t="inlineStr">
+        <is>
+          <t>Maximo Encarnacion</t>
+        </is>
+      </c>
+      <c r="E72" s="21" t="n">
+        <v>46207</v>
+      </c>
+      <c r="F72" s="22" t="n">
+        <v>9</v>
+      </c>
+      <c r="G72" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H72" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I72" s="14" t="inlineStr"/>
+      <c r="J72" s="15" t="inlineStr">
+        <is>
+          <t>Reclamo</t>
+        </is>
+      </c>
+      <c r="K72" s="15" t="inlineStr">
+        <is>
+          <t>Verificado: SALDO=0, CANCELADO, sin deuda pendiente.</t>
+        </is>
+      </c>
+      <c r="L72" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M72" s="17" t="inlineStr"/>
+      <c r="N72" s="18" t="n"/>
+      <c r="O72" s="18" t="n"/>
+      <c r="P72" s="23" t="n">
+        <v>46227.61004721065</v>
+      </c>
+      <c r="Q72" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R72" s="23" t="n">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="8" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B73" s="8" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C73" s="9" t="inlineStr">
+        <is>
+          <t>mesa_4</t>
+        </is>
+      </c>
+      <c r="D73" s="10" t="inlineStr">
+        <is>
+          <t>Wagner Trujillo</t>
+        </is>
+      </c>
+      <c r="E73" s="21" t="n">
+        <v>46208</v>
+      </c>
+      <c r="F73" s="22" t="n">
+        <v>53</v>
+      </c>
+      <c r="G73" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H73" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I73" s="14" t="inlineStr">
+        <is>
+          <t>convenio</t>
+        </is>
+      </c>
+      <c r="J73" s="15" t="inlineStr">
+        <is>
+          <t>Reclamo. Revisar medidor</t>
+        </is>
+      </c>
+      <c r="K73" s="15" t="inlineStr">
+        <is>
+          <t>Confirmado: pago de junio retenido por el cobrador (yape a cuenta personal), recuperado y aplicado via shared/abonos_rezagados.xlsx. SALDO=0 CANCELADO, incluido el medidor.</t>
+        </is>
+      </c>
+      <c r="L73" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M73" s="17" t="inlineStr"/>
+      <c r="N73" s="18" t="n"/>
+      <c r="O73" s="18" t="n"/>
+      <c r="P73" s="23" t="n">
+        <v>46227.61004721065</v>
+      </c>
+      <c r="Q73" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R73" s="23" t="n">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B74" s="8" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C74" s="9" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="D74" s="10" t="inlineStr">
+        <is>
+          <t>Secretaria</t>
+        </is>
+      </c>
+      <c r="E74" s="21" t="n"/>
+      <c r="F74" s="22" t="n"/>
+      <c r="G74" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H74" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I74" s="14" t="inlineStr"/>
+      <c r="J74" s="15" t="inlineStr">
+        <is>
+          <t>Actualizar Iglesia Bautista. Tiene que salir a nombre de Ramos Requez Mendoza es M-12. Pago 266, pago hasta octubre 25 este mes vendra consumo total lo que le resta hasta la fecha. Multa, faena, reunion, etc.</t>
+        </is>
+      </c>
+      <c r="K74" s="15" t="inlineStr">
+        <is>
+          <t>Corregido via overrides_padron.xlsx (0_padron) — CORREGIR_CAMPO NOMBRE, vigente 2026-08 (compra de lote, acuerdo entre ambos, no reasignacion). No es un TIPO_RECLAMO de deuda, es identidad del padron.</t>
+        </is>
+      </c>
+      <c r="L74" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M74" s="17" t="inlineStr"/>
+      <c r="N74" s="18" t="n"/>
+      <c r="O74" s="18" t="n"/>
+      <c r="P74" s="23" t="n">
+        <v>46225</v>
+      </c>
+      <c r="Q74" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R74" s="23" t="n">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="B75" s="8" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C75" s="9" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="D75" s="10" t="inlineStr"/>
+      <c r="E75" s="21" t="n"/>
+      <c r="F75" s="22" t="n"/>
+      <c r="G75" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H75" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I75" s="14" t="inlineStr"/>
+      <c r="J75" s="15" t="inlineStr">
+        <is>
+          <t>Flor Valdivia resta 350 por instalacion mas consumo</t>
+        </is>
+      </c>
+      <c r="K75" s="15" t="inlineStr"/>
+      <c r="L75" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M75" s="17" t="inlineStr"/>
+      <c r="N75" s="18" t="n"/>
+      <c r="O75" s="18" t="n"/>
+      <c r="P75" s="23" t="n"/>
+      <c r="Q75" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R75" s="23" t="n">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="8" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="B76" s="8" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C76" s="9" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="D76" s="10" t="inlineStr">
+        <is>
+          <t>Yanet Villanueva</t>
+        </is>
+      </c>
+      <c r="E76" s="21" t="n">
+        <v>46216</v>
+      </c>
+      <c r="F76" s="22" t="n"/>
+      <c r="G76" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H76" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I76" s="14" t="inlineStr"/>
+      <c r="J76" s="15" t="inlineStr">
+        <is>
+          <t>Nombre incorrecto: F1-6 es Viru Gaspar (esta al dia, yapeo su corte 20 adelantado), no Gaspar solo. [13/7/2026 12:07 y repetido 20/7/2026 10:20]</t>
+        </is>
+      </c>
+      <c r="K76" s="15" t="inlineStr">
+        <is>
+          <t>Corregido via overrides_padron.xlsx (0_padron) — CORREGIR_CAMPO NOMBRE F1-6=VIRU GASPAR, vigente 2026-08. Padron tenia el nombre invertido con F1-7, confirmado por el dato real.</t>
+        </is>
+      </c>
+      <c r="L76" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M76" s="17" t="inlineStr"/>
+      <c r="N76" s="18" t="n"/>
+      <c r="O76" s="18" t="n"/>
+      <c r="P76" s="23" t="n">
+        <v>46225</v>
+      </c>
+      <c r="Q76" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R76" s="23" t="n">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="8" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="B77" s="8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C77" s="9" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="D77" s="10" t="inlineStr">
+        <is>
+          <t>Yanet Villanueva</t>
+        </is>
+      </c>
+      <c r="E77" s="21" t="n">
+        <v>46216</v>
+      </c>
+      <c r="F77" s="22" t="n"/>
+      <c r="G77" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H77" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I77" s="14" t="inlineStr"/>
+      <c r="J77" s="15" t="inlineStr">
+        <is>
+          <t>Nombre incorrecto: F1-7 es Candacho (ya vino a pagar). [13/7/2026 12:07 y repetido 20/7/2026 10:20]</t>
+        </is>
+      </c>
+      <c r="K77" s="15" t="inlineStr">
+        <is>
+          <t>Corregido via overrides_padron.xlsx (0_padron) — CORREGIR_CAMPO NOMBRE F1-7=CANDACHO, vigente 2026-08. Padron tenia el nombre invertido con F1-6, confirmado por el dato real.</t>
+        </is>
+      </c>
+      <c r="L77" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M77" s="17" t="inlineStr"/>
+      <c r="N77" s="18" t="n"/>
+      <c r="O77" s="18" t="n"/>
+      <c r="P77" s="23" t="n">
+        <v>46225</v>
+      </c>
+      <c r="Q77" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R77" s="23" t="n">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="8" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="B78" s="8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C78" s="9" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="D78" s="10" t="inlineStr">
+        <is>
+          <t>Yanet Villanueva</t>
+        </is>
+      </c>
+      <c r="E78" s="21" t="n">
+        <v>46219</v>
+      </c>
+      <c r="F78" s="22" t="n"/>
+      <c r="G78" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H78" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I78" s="14" t="inlineStr"/>
+      <c r="J78" s="15" t="inlineStr">
+        <is>
+          <t>Pago efectivo 101 (no corresponde corte). Recibo trae 180 de la vez pasada; correcto: resta 50 + consumo 26 + mantenimiento 3 = deuda total 79 solo de este mes. [16/7/2026 22:17]</t>
+        </is>
+      </c>
+      <c r="K78" s="15" t="inlineStr"/>
+      <c r="L78" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M78" s="17" t="inlineStr"/>
+      <c r="N78" s="18" t="n"/>
+      <c r="O78" s="18" t="n"/>
+      <c r="P78" s="23" t="n"/>
+      <c r="Q78" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R78" s="23" t="n">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="8" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B79" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C79" s="9" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="D79" s="10" t="inlineStr">
+        <is>
+          <t>Janet Villanueva Alegre</t>
+        </is>
+      </c>
+      <c r="E79" s="21" t="n">
+        <v>46217</v>
+      </c>
+      <c r="F79" s="22" t="n"/>
+      <c r="G79" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H79" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I79" s="14" t="inlineStr"/>
+      <c r="J79" s="15" t="inlineStr">
+        <is>
+          <t>Yape de 30 quedo mal tipeado como D1-1; es D1-3 de Margarita Criollo. Actualizar. [14/7/2026 14:35, WhatsApp janetvillanuevaalegre]</t>
+        </is>
+      </c>
+      <c r="K79" s="15" t="inlineStr"/>
+      <c r="L79" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M79" s="17" t="inlineStr"/>
+      <c r="N79" s="18" t="n"/>
+      <c r="O79" s="18" t="n"/>
+      <c r="P79" s="23" t="n"/>
+      <c r="Q79" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R79" s="23" t="n">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B80" s="8" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C80" s="9" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="D80" s="10" t="inlineStr">
+        <is>
+          <t>Yanet Villanueva</t>
+        </is>
+      </c>
+      <c r="E80" s="21" t="n">
+        <v>46217</v>
+      </c>
+      <c r="F80" s="22" t="n"/>
+      <c r="G80" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H80" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I80" s="14" t="inlineStr"/>
+      <c r="J80" s="15" t="inlineStr">
+        <is>
+          <t>No se encontro su pago (David / 'nena' Chinchay). Wagner confirma: solo pago consumo mes anterior + mes actual, agregar resto como compromiso de pago este mes. [14/7/2026 05:44-07:45]</t>
+        </is>
+      </c>
+      <c r="K80" s="15" t="inlineStr"/>
+      <c r="L80" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M80" s="17" t="inlineStr"/>
+      <c r="N80" s="18" t="n"/>
+      <c r="O80" s="18" t="n"/>
+      <c r="P80" s="23" t="n"/>
+      <c r="Q80" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R80" s="23" t="n">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="8" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B81" s="8" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="C81" s="9" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="D81" s="10" t="inlineStr">
+        <is>
+          <t>Janet Villanueva Alegre</t>
+        </is>
+      </c>
+      <c r="E81" s="21" t="n">
+        <v>46217</v>
+      </c>
+      <c r="F81" s="22" t="n"/>
+      <c r="G81" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H81" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I81" s="14" t="inlineStr"/>
+      <c r="J81" s="15" t="inlineStr">
+        <is>
+          <t>Hasta el momento no debe nada, conversado con ella, pagos al dia -&gt; borrar del corte. [14/7/2026 14:47, WhatsApp janetvillanuevaalegre]</t>
+        </is>
+      </c>
+      <c r="K81" s="15" t="inlineStr"/>
+      <c r="L81" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M81" s="17" t="inlineStr"/>
+      <c r="N81" s="18" t="n"/>
+      <c r="O81" s="18" t="n"/>
+      <c r="P81" s="23" t="n"/>
+      <c r="Q81" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R81" s="23" t="n">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="8" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B82" s="8" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="C82" s="9" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="D82" s="10" t="inlineStr">
+        <is>
+          <t>Yanet Villanueva</t>
+        </is>
+      </c>
+      <c r="E82" s="21" t="n">
+        <v>46218</v>
+      </c>
+      <c r="F82" s="22" t="n"/>
+      <c r="G82" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H82" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I82" s="14" t="inlineStr"/>
+      <c r="J82" s="15" t="inlineStr">
+        <is>
+          <t>Sr. Hipolito Ramirez: su hijo fue a pagar incluyendo las multas -&gt; sacar de la lista de corte. [15/7/2026 06:55-08:52]</t>
+        </is>
+      </c>
+      <c r="K82" s="15" t="inlineStr"/>
+      <c r="L82" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M82" s="17" t="inlineStr"/>
+      <c r="N82" s="18" t="n"/>
+      <c r="O82" s="18" t="n"/>
+      <c r="P82" s="23" t="n"/>
+      <c r="Q82" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R82" s="23" t="n">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="8" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B83" s="8" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C83" s="9" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="D83" s="10" t="inlineStr">
+        <is>
+          <t>Yanet Villanueva</t>
+        </is>
+      </c>
+      <c r="E83" s="21" t="n">
+        <v>46219</v>
+      </c>
+      <c r="F83" s="22" t="n"/>
+      <c r="G83" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H83" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I83" s="14" t="inlineStr"/>
+      <c r="J83" s="15" t="inlineStr">
+        <is>
+          <t>Pago su consumo, no entra a corte. Conversado con la vecina. [16/7/2026 08:19]</t>
+        </is>
+      </c>
+      <c r="K83" s="15" t="inlineStr">
+        <is>
+          <t>Pago S/86 (Yape, junio) retenido por el cobrador Wagner Trujillo, recuperado en efectivo y aplicado en julio (shared/abonos_rezagados.xlsx). MES_ANTERIOR/CORTE_RECONEXION/MULTA quedan en 0 tras el overlay - ya no cumple criterio de corte (MES_ANTERIOR&gt;=8). Confirmado, no aparece en lista_corte.xlsx ni registro_cortes.xlsx.</t>
+        </is>
+      </c>
+      <c r="L83" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M83" s="17" t="inlineStr"/>
+      <c r="N83" s="18" t="n"/>
+      <c r="O83" s="18" t="n"/>
+      <c r="P83" s="23" t="n">
+        <v>46227.40791967593</v>
+      </c>
+      <c r="Q83" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R83" s="23" t="n">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="8" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="B84" s="8" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C84" s="9" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="D84" s="10" t="inlineStr">
+        <is>
+          <t>Yanet Villanueva</t>
+        </is>
+      </c>
+      <c r="E84" s="21" t="n">
+        <v>46221</v>
+      </c>
+      <c r="F84" s="22" t="n"/>
+      <c r="G84" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H84" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I84" s="14" t="inlineStr"/>
+      <c r="J84" s="15" t="inlineStr">
+        <is>
+          <t>Sra. Teodora Meza Garcilazo: pago 50 el mes anterior segun hoja del Sr. Maximo. OJO: memoria de sesion previa registra este caso como Q-6, verificar cual MZ es correcta antes de aplicar. [18/7/2026 16:21]</t>
+        </is>
+      </c>
+      <c r="K84" s="15" t="inlineStr">
+        <is>
+          <t>El pago de S/50 (Maximo Encarnacion, mesa_5, 05/06/2026, registrado como blanco) es aporte voluntario a tanque (shared/aportes_tanque_manuales.xlsx), NO pago de deuda. Su agua de junio (15) ya estaba cubierta por otro pago (Wagner Trujillo, mesa_6, mismo dia). Su MULTA=30 sigue pendiente, sin relacion con este aporte.</t>
+        </is>
+      </c>
+      <c r="L84" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M84" s="17" t="inlineStr"/>
+      <c r="N84" s="18" t="n"/>
+      <c r="O84" s="18" t="n"/>
+      <c r="P84" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="Q84" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R84" s="23" t="n">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="8" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B85" s="8" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C85" s="9" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="D85" s="10" t="inlineStr">
+        <is>
+          <t>Yanet Villanueva</t>
+        </is>
+      </c>
+      <c r="E85" s="21" t="n">
+        <v>46221</v>
+      </c>
+      <c r="F85" s="22" t="n"/>
+      <c r="G85" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H85" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I85" s="14" t="inlineStr"/>
+      <c r="J85" s="15" t="inlineStr">
+        <is>
+          <t>Esta al dia, solo debe consumo de este mes. [18/7/2026 22:16]</t>
+        </is>
+      </c>
+      <c r="K85" s="15" t="inlineStr"/>
+      <c r="L85" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M85" s="17" t="inlineStr"/>
+      <c r="N85" s="18" t="n"/>
+      <c r="O85" s="18" t="n"/>
+      <c r="P85" s="23" t="n"/>
+      <c r="Q85" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R85" s="23" t="n">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="8" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B86" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C86" s="9" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="D86" s="10" t="inlineStr">
+        <is>
+          <t>Yanet Villanueva</t>
+        </is>
+      </c>
+      <c r="E86" s="21" t="n">
+        <v>46216</v>
+      </c>
+      <c r="F86" s="22" t="n"/>
+      <c r="G86" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H86" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I86" s="14" t="inlineStr"/>
+      <c r="J86" s="15" t="inlineStr">
+        <is>
+          <t>Sacar de lista de corte (junto con B-19 y D1-3); revisar con hoja del gringo si llego a anotar su yape. [13/7/2026 12:07-16:14]</t>
+        </is>
+      </c>
+      <c r="K86" s="15" t="inlineStr"/>
+      <c r="L86" s="16" t="inlineStr">
+        <is>
+          <t>RESUELTO</t>
+        </is>
+      </c>
+      <c r="M86" s="17" t="inlineStr"/>
+      <c r="N86" s="18" t="n"/>
+      <c r="O86" s="18" t="n"/>
+      <c r="P86" s="23" t="n"/>
+      <c r="Q86" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R86" s="23" t="n">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="D87" s="10" t="inlineStr">
+        <is>
+          <t>Secretaria</t>
+        </is>
+      </c>
+      <c r="E87" s="21" t="n"/>
+      <c r="F87" s="22" t="n"/>
+      <c r="G87" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H87" s="13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I87" s="14" t="inlineStr">
+        <is>
+          <t>cuota</t>
+        </is>
+      </c>
+      <c r="J87" s="15" t="inlineStr">
+        <is>
+          <t>Por que aun debe S/30 de techado y campo?</t>
+        </is>
+      </c>
+      <c r="K87" s="15" t="inlineStr">
+        <is>
+          <t>Deuda legitima. Debia S/50 de acuerdos (techado+campo), va pagando en cuotas (S/10/mes): pago 20, saldo real S/30 pendiente. No hay error de cobro. Aparte tiene S/75 a favor en convenio (medidor, pago de mas en abril-mayo antes del ledger) que no se cruza automaticamente con acuerdos. Informar a la senora; si reclama, evaluar aplicar ese exceso contra este saldo.</t>
+        </is>
+      </c>
+      <c r="L87" s="16" t="inlineStr">
+        <is>
+          <t>INFORMADO</t>
+        </is>
+      </c>
+      <c r="M87" s="17" t="inlineStr">
+        <is>
+          <t>Cuota directa</t>
+        </is>
+      </c>
+      <c r="N87" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="O87" s="18" t="n"/>
+      <c r="P87" s="23" t="n">
+        <v>46231</v>
+      </c>
+      <c r="Q87" s="20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="R87" s="23" t="n">
+        <v>46231</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="J1:L1"/>

</xml_diff>